<commit_message>
feat: cc4k downloadable tree
</commit_message>
<xml_diff>
--- a/public/files/cc4k/Official_CC4K_v0.5.2.xlsx
+++ b/public/files/cc4k/Official_CC4K_v0.5.2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mkirk/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mkirk/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5C6AB60B-C1CF-E949-8BE0-7A90900886CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{74E82519-3A06-164B-9761-5AAA6795CC73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="840" yWindow="1520" windowWidth="29400" windowHeight="16440" firstSheet="1" activeTab="1" xr2:uid="{924538EB-B3B0-A84F-847F-99AE6552E62D}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" firstSheet="1" activeTab="2" xr2:uid="{924538EB-B3B0-A84F-847F-99AE6552E62D}"/>
   </bookViews>
   <sheets>
     <sheet name="OntologyList v0.5.2" sheetId="8" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5029" uniqueCount="1068">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5030" uniqueCount="1068">
   <si>
     <t>disease_name</t>
   </si>
@@ -15729,7 +15729,9 @@
       <c r="C1" s="792"/>
       <c r="D1" s="792"/>
       <c r="E1" s="24"/>
-      <c r="F1" s="25"/>
+      <c r="F1" s="25" t="s">
+        <v>1047</v>
+      </c>
       <c r="G1" s="25" t="s">
         <v>1029</v>
       </c>
@@ -17591,7 +17593,7 @@
         <v>86</v>
       </c>
       <c r="G82" s="198" t="s">
-        <v>818</v>
+        <v>87</v>
       </c>
       <c r="H82" s="240" t="s">
         <v>1032</v>
@@ -27141,6 +27143,28 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="2936e93f-eedd-41e3-9791-66a5f5ce8353" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ff0e03ee-7665-4114-9abd-caa5292aa2b1">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100401465C67862AF44974A5795FB7A315A" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="53103cc66cf7492b1d451bf4d1d198c3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="ff0e03ee-7665-4114-9abd-caa5292aa2b1" xmlns:ns3="2936e93f-eedd-41e3-9791-66a5f5ce8353" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="16821dee0b9fa2cb8b7ea0abefb318c2" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -27412,29 +27436,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <TaxCatchAll xmlns="2936e93f-eedd-41e3-9791-66a5f5ce8353" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ff0e03ee-7665-4114-9abd-caa5292aa2b1">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A6A7D65-2E6B-4214-A9A5-86974DA224D3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1722472A-1E8F-4733-8990-41D115C3D7F9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="2936e93f-eedd-41e3-9791-66a5f5ce8353"/>
+    <ds:schemaRef ds:uri="ff0e03ee-7665-4114-9abd-caa5292aa2b1"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9766029B-62D1-4923-8FF5-D469D306FA99}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -27454,26 +27476,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1722472A-1E8F-4733-8990-41D115C3D7F9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="2936e93f-eedd-41e3-9791-66a5f5ce8353"/>
-    <ds:schemaRef ds:uri="ff0e03ee-7665-4114-9abd-caa5292aa2b1"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A6A7D65-2E6B-4214-A9A5-86974DA224D3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{65ce1208-e929-4ec4-be64-9138d78922c0}" enabled="1" method="Standard" siteId="{22340fa8-9226-4871-b677-d3b3e377af72}" contentBits="2" removed="0"/>

</xml_diff>